<commit_message>
Release v0.2.0: NVL authoring, project launcher and four-language workflow improvements
</commit_message>
<xml_diff>
--- a/examples/localized/en/branches.xlsx
+++ b/examples/localized/en/branches.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -728,6 +728,11 @@
           <t>顏色</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>文字模式</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -745,6 +750,11 @@
           <t>#e5b5a5</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>adv</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -760,6 +770,11 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>#b0c9ed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>adv</t>
         </is>
       </c>
     </row>

</xml_diff>